<commit_message>
changes to the schedule of events- Pre proposal
</commit_message>
<xml_diff>
--- a/Oversight-AYAC 2026 Schedule.xlsx
+++ b/Oversight-AYAC 2026 Schedule.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6a43dedaebc80f39/Documents/WCIE/AYAC/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Israel Adefemi\Documents\Office\AYAC 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="118" documentId="8_{0CFFD51D-F4F0-42C7-98D8-F1B1C621522F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9F0BDD0-B104-4C6B-846D-6DD9D9FF2E01}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{318D0133-DB75-4569-82AC-4FF5BD536B23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E09745D3-EC13-3B4E-8089-EA3CE444E0AC}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{E09745D3-EC13-3B4E-8089-EA3CE444E0AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Schedule" sheetId="2" r:id="rId1"/>
@@ -440,13 +440,19 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -640,108 +646,108 @@
   </cellStyleXfs>
   <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -764,10 +770,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1091,67 +1093,67 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="C3:O38"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="9.1796875" style="1"/>
+    <col min="1" max="2" width="9.140625" style="1"/>
     <col min="3" max="3" width="19" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="19.54296875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="23.81640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="23.54296875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="51.26953125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="21.54296875" style="1" customWidth="1"/>
-    <col min="11" max="12" width="29.81640625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="26.453125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="33.1796875" style="1" customWidth="1"/>
-    <col min="15" max="15" width="18.1796875" style="1" customWidth="1"/>
-    <col min="16" max="19" width="9.1796875" style="1"/>
-    <col min="20" max="20" width="33.54296875" style="1" customWidth="1"/>
-    <col min="21" max="16384" width="9.1796875" style="1"/>
+    <col min="4" max="6" width="19.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="23.85546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="23.5703125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="51.28515625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="21.5703125" style="1" customWidth="1"/>
+    <col min="11" max="12" width="29.85546875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="26.42578125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="33.140625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="18.140625" style="1" customWidth="1"/>
+    <col min="16" max="19" width="9.140625" style="1"/>
+    <col min="20" max="20" width="33.5703125" style="1" customWidth="1"/>
+    <col min="21" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:15" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="24" t="s">
+    <row r="3" spans="3:15" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C3" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-      <c r="M3" s="24"/>
-      <c r="N3" s="24"/>
-      <c r="O3" s="24"/>
-    </row>
-    <row r="4" spans="3:15" ht="31" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="22"/>
+      <c r="O3" s="22"/>
+    </row>
+    <row r="4" spans="3:15" ht="30.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="31" t="s">
+      <c r="D4" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="H4" s="31"/>
-      <c r="I4" s="31" t="s">
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="31"/>
-      <c r="K4" s="31"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
       <c r="L4" s="11"/>
-      <c r="M4" s="31" t="s">
+      <c r="M4" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="N4" s="31"/>
+      <c r="N4" s="27"/>
       <c r="O4" s="11" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="3:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:15" ht="41.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C5" s="4"/>
       <c r="D5" s="7" t="s">
         <v>6</v>
@@ -1180,65 +1182,65 @@
       <c r="L5" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="M5" s="16" t="s">
+      <c r="M5" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="N5" s="17"/>
+      <c r="N5" s="31"/>
       <c r="O5" s="13"/>
     </row>
-    <row r="6" spans="3:15" ht="28" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:15" ht="27.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="18" t="s">
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="25"/>
+      <c r="J6" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="32"/>
       <c r="M6" s="12" t="s">
         <v>68</v>
       </c>
       <c r="N6" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="O6" s="27" t="s">
+      <c r="O6" s="17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="3:15" ht="141" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C7" s="25" t="s">
+    <row r="7" spans="3:15" ht="141" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C7" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="28" t="s">
+      <c r="D7" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="27" t="s">
+      <c r="E7" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="35" t="s">
+      <c r="F7" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="G7" s="26" t="s">
+      <c r="G7" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="H7" s="30" t="s">
+      <c r="H7" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="I7" s="26" t="s">
+      <c r="I7" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="J7" s="27" t="s">
+      <c r="J7" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="K7" s="26" t="s">
+      <c r="K7" s="20" t="s">
         <v>17</v>
       </c>
       <c r="L7" s="14" t="s">
@@ -1250,108 +1252,108 @@
       <c r="N7" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="O7" s="27"/>
-    </row>
-    <row r="8" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="C8" s="25"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="26"/>
-      <c r="J8" s="27"/>
-      <c r="K8" s="26"/>
+      <c r="O7" s="17"/>
+    </row>
+    <row r="8" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="C8" s="23"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="20"/>
       <c r="L8" s="15"/>
       <c r="M8" s="6"/>
       <c r="N8" s="6"/>
-      <c r="O8" s="27"/>
-    </row>
-    <row r="9" spans="3:15" ht="141" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="25" t="s">
+      <c r="O8" s="17"/>
+    </row>
+    <row r="9" spans="3:15" ht="141" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C9" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="28"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="26" t="s">
+      <c r="D9" s="24"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="H9" s="30"/>
-      <c r="I9" s="26"/>
-      <c r="J9" s="27"/>
-      <c r="K9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="20"/>
       <c r="L9" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="M9" s="20" t="s">
+      <c r="M9" s="33" t="s">
         <v>69</v>
       </c>
-      <c r="N9" s="21"/>
-      <c r="O9" s="27"/>
-    </row>
-    <row r="10" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="C10" s="25"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="27"/>
-      <c r="K10" s="26"/>
+      <c r="N9" s="34"/>
+      <c r="O9" s="17"/>
+    </row>
+    <row r="10" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="C10" s="23"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="20"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="20"/>
       <c r="L10" s="15"/>
       <c r="M10" s="6"/>
       <c r="N10" s="6"/>
-      <c r="O10" s="27"/>
-    </row>
-    <row r="11" spans="3:15" ht="136.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O10" s="17"/>
+    </row>
+    <row r="11" spans="3:15" ht="136.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="28"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="35"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="21"/>
       <c r="G11" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="H11" s="30"/>
+      <c r="H11" s="26"/>
       <c r="I11" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="J11" s="27"/>
-      <c r="K11" s="26"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="20"/>
       <c r="L11" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="M11" s="26" t="s">
+      <c r="M11" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="N11" s="26"/>
-      <c r="O11" s="27"/>
-    </row>
-    <row r="12" spans="3:15" ht="128.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N11" s="20"/>
+      <c r="O11" s="17"/>
+    </row>
+    <row r="12" spans="3:15" ht="128.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C12" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="33" t="s">
+      <c r="D12" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="33"/>
-      <c r="F12" s="33"/>
-      <c r="G12" s="33"/>
-      <c r="H12" s="33"/>
-      <c r="I12" s="33"/>
-      <c r="J12" s="34" t="s">
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="K12" s="34"/>
-      <c r="L12" s="34"/>
-      <c r="M12" s="34"/>
-      <c r="N12" s="34"/>
-      <c r="O12" s="34"/>
-    </row>
-    <row r="16" spans="3:15" ht="28" x14ac:dyDescent="0.3">
+      <c r="K12" s="19"/>
+      <c r="L12" s="19"/>
+      <c r="M12" s="19"/>
+      <c r="N12" s="19"/>
+      <c r="O12" s="19"/>
+    </row>
+    <row r="16" spans="3:15" ht="30" x14ac:dyDescent="0.25">
       <c r="C16" s="3" t="s">
         <v>23</v>
       </c>
@@ -1360,11 +1362,11 @@
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
-      <c r="G16" s="32" t="s">
+      <c r="G16" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="H16" s="32"/>
-      <c r="I16" s="32"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
       <c r="J16" s="8"/>
       <c r="K16" s="8"/>
       <c r="L16" s="8"/>
@@ -1372,7 +1374,7 @@
       <c r="N16" s="8"/>
       <c r="O16" s="8"/>
     </row>
-    <row r="17" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:10" ht="15" x14ac:dyDescent="0.25">
       <c r="C17" s="9" t="s">
         <v>26</v>
       </c>
@@ -1381,14 +1383,14 @@
       </c>
       <c r="E17" s="8"/>
       <c r="F17" s="8"/>
-      <c r="G17" s="23" t="s">
+      <c r="G17" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="H17" s="23"/>
-      <c r="I17" s="23"/>
+      <c r="H17" s="29"/>
+      <c r="I17" s="29"/>
       <c r="J17" s="10"/>
     </row>
-    <row r="18" spans="3:10" ht="28" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="C18" s="9" t="s">
         <v>29</v>
       </c>
@@ -1397,14 +1399,14 @@
       </c>
       <c r="E18" s="8"/>
       <c r="F18" s="8"/>
-      <c r="G18" s="22" t="s">
+      <c r="G18" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="28"/>
       <c r="J18" s="10"/>
     </row>
-    <row r="19" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:10" ht="15" x14ac:dyDescent="0.25">
       <c r="C19" s="9" t="s">
         <v>32</v>
       </c>
@@ -1413,158 +1415,158 @@
       </c>
       <c r="E19" s="8"/>
       <c r="F19" s="8"/>
-      <c r="G19" s="23" t="s">
+      <c r="G19" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="H19" s="23"/>
-      <c r="I19" s="23"/>
+      <c r="H19" s="29"/>
+      <c r="I19" s="29"/>
       <c r="J19" s="10"/>
     </row>
-    <row r="20" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C20" s="8"/>
       <c r="D20" s="8"/>
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
-      <c r="G20" s="22" t="s">
+      <c r="G20" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="H20" s="22"/>
-      <c r="I20" s="22"/>
+      <c r="H20" s="28"/>
+      <c r="I20" s="28"/>
       <c r="J20" s="10"/>
     </row>
-    <row r="21" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C21" s="8"/>
       <c r="D21" s="8"/>
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
-      <c r="G21" s="22" t="s">
+      <c r="G21" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="H21" s="22"/>
-      <c r="I21" s="22"/>
+      <c r="H21" s="28"/>
+      <c r="I21" s="28"/>
       <c r="J21" s="10"/>
     </row>
-    <row r="22" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
-      <c r="G22" s="22" t="s">
+      <c r="G22" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="H22" s="22"/>
-      <c r="I22" s="22"/>
+      <c r="H22" s="28"/>
+      <c r="I22" s="28"/>
       <c r="J22" s="10"/>
     </row>
-    <row r="23" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C23" s="8"/>
       <c r="D23" s="8"/>
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
-      <c r="G23" s="22" t="s">
+      <c r="G23" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="H23" s="22"/>
-      <c r="I23" s="22"/>
+      <c r="H23" s="28"/>
+      <c r="I23" s="28"/>
       <c r="J23" s="10"/>
     </row>
-    <row r="24" spans="3:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C24" s="8"/>
       <c r="D24" s="8"/>
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
-      <c r="G24" s="22" t="s">
+      <c r="G24" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="H24" s="22"/>
-      <c r="I24" s="22"/>
+      <c r="H24" s="28"/>
+      <c r="I24" s="28"/>
       <c r="J24" s="10"/>
     </row>
-    <row r="25" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
-      <c r="G25" s="22" t="s">
+      <c r="G25" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="H25" s="22"/>
-      <c r="I25" s="22"/>
+      <c r="H25" s="28"/>
+      <c r="I25" s="28"/>
       <c r="J25" s="10"/>
     </row>
-    <row r="26" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C26" s="8"/>
       <c r="D26" s="8"/>
       <c r="E26" s="8"/>
       <c r="F26" s="8"/>
-      <c r="G26" s="22" t="s">
+      <c r="G26" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="H26" s="22"/>
-      <c r="I26" s="22"/>
+      <c r="H26" s="28"/>
+      <c r="I26" s="28"/>
       <c r="J26" s="10"/>
     </row>
-    <row r="27" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C27" s="8"/>
       <c r="D27" s="8"/>
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
-      <c r="G27" s="22" t="s">
+      <c r="G27" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="H27" s="22"/>
-      <c r="I27" s="22"/>
+      <c r="H27" s="28"/>
+      <c r="I27" s="28"/>
       <c r="J27" s="10"/>
     </row>
-    <row r="28" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:10" ht="15" x14ac:dyDescent="0.25">
       <c r="C28" s="8"/>
       <c r="D28" s="8"/>
       <c r="E28" s="8"/>
       <c r="F28" s="8"/>
-      <c r="G28" s="23" t="s">
+      <c r="G28" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="H28" s="23"/>
-      <c r="I28" s="23"/>
+      <c r="H28" s="29"/>
+      <c r="I28" s="29"/>
       <c r="J28" s="10"/>
     </row>
-    <row r="29" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C29" s="8"/>
       <c r="D29" s="8"/>
       <c r="E29" s="8"/>
       <c r="F29" s="8"/>
-      <c r="G29" s="22" t="s">
+      <c r="G29" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="H29" s="22"/>
-      <c r="I29" s="22"/>
+      <c r="H29" s="28"/>
+      <c r="I29" s="28"/>
       <c r="J29" s="10"/>
     </row>
-    <row r="30" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C30" s="8"/>
       <c r="D30" s="8"/>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
-      <c r="G30" s="22" t="s">
+      <c r="G30" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="H30" s="22"/>
-      <c r="I30" s="22"/>
+      <c r="H30" s="28"/>
+      <c r="I30" s="28"/>
       <c r="J30" s="10"/>
     </row>
-    <row r="31" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
-      <c r="G31" s="22" t="s">
+      <c r="G31" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="H31" s="22"/>
-      <c r="I31" s="22"/>
+      <c r="H31" s="28"/>
+      <c r="I31" s="28"/>
       <c r="J31" s="10"/>
     </row>
-    <row r="32" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C32" s="8"/>
       <c r="D32" s="8"/>
       <c r="E32" s="8"/>
@@ -1574,52 +1576,69 @@
       <c r="I32" s="8"/>
       <c r="J32" s="10"/>
     </row>
-    <row r="33" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G33" s="23" t="s">
+    <row r="33" spans="7:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="G33" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="H33" s="23"/>
-      <c r="I33" s="23"/>
-    </row>
-    <row r="34" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G34" s="22" t="s">
+      <c r="H33" s="29"/>
+      <c r="I33" s="29"/>
+    </row>
+    <row r="34" spans="7:9" x14ac:dyDescent="0.2">
+      <c r="G34" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="H34" s="22"/>
-      <c r="I34" s="22"/>
-    </row>
-    <row r="35" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G35" s="22" t="s">
+      <c r="H34" s="28"/>
+      <c r="I34" s="28"/>
+    </row>
+    <row r="35" spans="7:9" x14ac:dyDescent="0.2">
+      <c r="G35" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="H35" s="22"/>
-      <c r="I35" s="22"/>
-    </row>
-    <row r="36" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G36" s="22" t="s">
+      <c r="H35" s="28"/>
+      <c r="I35" s="28"/>
+    </row>
+    <row r="36" spans="7:9" x14ac:dyDescent="0.2">
+      <c r="G36" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="H36" s="22"/>
-      <c r="I36" s="22"/>
-    </row>
-    <row r="37" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G37" s="22"/>
-      <c r="H37" s="22"/>
-      <c r="I37" s="22"/>
-    </row>
-    <row r="38" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G38" s="22"/>
-      <c r="H38" s="22"/>
-      <c r="I38" s="22"/>
+      <c r="H36" s="28"/>
+      <c r="I36" s="28"/>
+    </row>
+    <row r="37" spans="7:9" x14ac:dyDescent="0.2">
+      <c r="G37" s="28"/>
+      <c r="H37" s="28"/>
+      <c r="I37" s="28"/>
+    </row>
+    <row r="38" spans="7:9" x14ac:dyDescent="0.2">
+      <c r="G38" s="28"/>
+      <c r="H38" s="28"/>
+      <c r="I38" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="45">
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="E7:E11"/>
-    <mergeCell ref="D12:I12"/>
-    <mergeCell ref="J12:O12"/>
-    <mergeCell ref="M11:N11"/>
-    <mergeCell ref="F7:F11"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="G38:I38"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="G34:I34"/>
+    <mergeCell ref="G35:I35"/>
+    <mergeCell ref="G36:I36"/>
+    <mergeCell ref="G37:I37"/>
+    <mergeCell ref="G28:I28"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="G22:I22"/>
     <mergeCell ref="C3:O3"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="C9:C10"/>
@@ -1635,32 +1654,15 @@
     <mergeCell ref="M4:N4"/>
     <mergeCell ref="D4:H4"/>
     <mergeCell ref="I4:K4"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="G21:I21"/>
-    <mergeCell ref="G22:I22"/>
     <mergeCell ref="M5:N5"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="G38:I38"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="G34:I34"/>
-    <mergeCell ref="G35:I35"/>
-    <mergeCell ref="G36:I36"/>
-    <mergeCell ref="G37:I37"/>
-    <mergeCell ref="G28:I28"/>
-    <mergeCell ref="G29:I29"/>
-    <mergeCell ref="G30:I30"/>
-    <mergeCell ref="G31:I31"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="E7:E11"/>
+    <mergeCell ref="D12:I12"/>
+    <mergeCell ref="J12:O12"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="F7:F11"/>
   </mergeCells>
-  <phoneticPr fontId="5" type="noConversion"/>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="34" orientation="landscape" r:id="rId1"/>
 </worksheet>

</xml_diff>